<commit_message>
fix: template README - CS1 長沙灣分校 (not 警察少年之家)
</commit_message>
<xml_diff>
--- a/api/template_v4.xlsx
+++ b/api/template_v4.xlsx
@@ -518,7 +518,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -637,7 +637,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>TW2 = 屯門分校第2組，CS1 = 長沙灣警察少年之家第1組</t>
+          <t>TW2 = 屯門分校第2組，CS1 = 長沙灣分校第1組</t>
         </is>
       </c>
     </row>
@@ -3323,11 +3323,11 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">

</xml_diff>

<commit_message>
feat(template): add CC Group column + docs to V4 templates
- Add a "CC Group" column to the Class list of both V4 templates
  (api/template_v4.xlsx served by the UI, and the data/input copy), styled to
  match the existing headers.
- Label three fully-present combine groups as live examples
  (CS6+WT2, TW1+TW3, TS1+TS2 -> CC-DAE106-1/2/3).
- Append a "分班 / 規則 (2026-08)" section to the READ ME sheet documenting the
  CC Group column, the DAE Mon/Tue/Thu day rule, and the loading soft cap.
- Script: scripts/update_template_cc_group.py.

Closes the gap where the combine feature had no template column and no READ ME
mention. Engine parse verified: the three example groups load correctly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/api/template_v4.xlsx
+++ b/api/template_v4.xlsx
@@ -119,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -151,6 +151,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -655,6 +656,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -683,6 +685,50 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>⭐ 留空則系統自動分配英文老師；只在想手動鎖定個別班時才填</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>分班 / 規則 (2026-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>CC Group 欄</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>要合併上課的班別填相同標籤（例：DAE106_CS6 與 DAE106_WT2 同填 CC-DAE106-1）；留空 = 不合併。只在 Class list answer 留空（自動排班）時生效。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>上課日</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DAE 科目只排 Mon / Tue / Thu（不排星期三、五）；Cadet 班維持 Mon / Wed / Fri。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>老師 Loading</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>每週建議上限 6 班；可超過，只會提醒不會阻擋（超出者在畫面標示紅色「超限」）。</t>
         </is>
       </c>
     </row>
@@ -697,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -705,6 +751,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -763,6 +810,11 @@
           <t>Date (optional)</t>
         </is>
       </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>CC Group</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2787,6 +2839,11 @@
       <c r="H89" t="n">
         <v>33</v>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>CC-DAE106-1</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2833,6 +2890,11 @@
       <c r="H91" t="n">
         <v>28</v>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>CC-DAE106-1</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2879,6 +2941,11 @@
       <c r="H93" t="n">
         <v>33</v>
       </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>CC-DAE106-2</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2925,6 +2992,11 @@
       <c r="H95" t="n">
         <v>23</v>
       </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>CC-DAE106-2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2994,6 +3066,11 @@
       <c r="H98" t="n">
         <v>20</v>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>CC-DAE106-3</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3016,6 +3093,11 @@
       </c>
       <c r="H99" t="n">
         <v>19</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>CC-DAE106-3</t>
+        </is>
       </c>
     </row>
     <row r="100">

</xml_diff>